<commit_message>
docs(middleware): clarify PTseq template inputs
</commit_message>
<xml_diff>
--- a/中台配置/GenSIRO48-PTseq/Resources/SIRO48_template.xlsx
+++ b/中台配置/GenSIRO48-PTseq/Resources/SIRO48_template.xlsx
@@ -1498,7 +1498,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
@@ -1698,39 +1698,13 @@
       </c>
     </row>
     <row r="4" ht="16.5" customFormat="1" customHeight="1" s="3">
-      <c r="A4" s="20" t="inlineStr">
-        <is>
-          <t>25S02270001</t>
-        </is>
-      </c>
-      <c r="B4" s="20" t="inlineStr">
-        <is>
-          <t>PTseq</t>
-        </is>
-      </c>
-      <c r="C4" s="20" t="inlineStr">
-        <is>
-          <t>100K</t>
-        </is>
-      </c>
-      <c r="D4" s="27" t="inlineStr">
-        <is>
-          <t>痰液</t>
-        </is>
-      </c>
-      <c r="E4" s="20" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F4" s="20" t="inlineStr">
-        <is>
-          <t>DNA+RNA</t>
-        </is>
-      </c>
-      <c r="G4" s="20" t="n">
-        <v>1</v>
-      </c>
+      <c r="A4" s="20" t="n"/>
+      <c r="B4" s="20" t="n"/>
+      <c r="C4" s="20" t="n"/>
+      <c r="D4" s="27" t="n"/>
+      <c r="E4" s="20" t="n"/>
+      <c r="F4" s="20" t="n"/>
+      <c r="G4" s="20" t="n"/>
       <c r="H4" s="20" t="n"/>
       <c r="I4" s="20" t="n"/>
       <c r="J4" s="20" t="n"/>
@@ -1763,39 +1737,13 @@
       <c r="AY4" s="20" t="n"/>
     </row>
     <row r="5" ht="16.5" customFormat="1" customHeight="1" s="3">
-      <c r="A5" s="20" t="inlineStr">
-        <is>
-          <t>25S02270002</t>
-        </is>
-      </c>
-      <c r="B5" s="20" t="inlineStr">
-        <is>
-          <t>PTseq</t>
-        </is>
-      </c>
-      <c r="C5" s="20" t="inlineStr">
-        <is>
-          <t>100K</t>
-        </is>
-      </c>
-      <c r="D5" s="27" t="inlineStr">
-        <is>
-          <t>肺泡灌洗液</t>
-        </is>
-      </c>
-      <c r="E5" s="20" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F5" s="20" t="inlineStr">
-        <is>
-          <t>DNA+RNA</t>
-        </is>
-      </c>
-      <c r="G5" s="20" t="n">
-        <v>2</v>
-      </c>
+      <c r="A5" s="20" t="n"/>
+      <c r="B5" s="20" t="n"/>
+      <c r="C5" s="20" t="n"/>
+      <c r="D5" s="27" t="n"/>
+      <c r="E5" s="20" t="n"/>
+      <c r="F5" s="20" t="n"/>
+      <c r="G5" s="20" t="n"/>
       <c r="H5" s="20" t="n"/>
       <c r="I5" s="20" t="n"/>
       <c r="J5" s="20" t="n"/>
@@ -1828,39 +1776,13 @@
       <c r="AY5" s="20" t="n"/>
     </row>
     <row r="6" ht="16.5" customFormat="1" customHeight="1" s="3">
-      <c r="A6" s="20" t="inlineStr">
-        <is>
-          <t>25S02270003</t>
-        </is>
-      </c>
-      <c r="B6" s="20" t="inlineStr">
-        <is>
-          <t>PTseq</t>
-        </is>
-      </c>
-      <c r="C6" s="20" t="inlineStr">
-        <is>
-          <t>100K</t>
-        </is>
-      </c>
-      <c r="D6" s="27" t="inlineStr">
-        <is>
-          <t>口咽拭子</t>
-        </is>
-      </c>
-      <c r="E6" s="20" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F6" s="20" t="inlineStr">
-        <is>
-          <t>DNA+RNA</t>
-        </is>
-      </c>
-      <c r="G6" s="20" t="n">
-        <v>5</v>
-      </c>
+      <c r="A6" s="20" t="n"/>
+      <c r="B6" s="20" t="n"/>
+      <c r="C6" s="20" t="n"/>
+      <c r="D6" s="27" t="n"/>
+      <c r="E6" s="20" t="n"/>
+      <c r="F6" s="20" t="n"/>
+      <c r="G6" s="20" t="n"/>
       <c r="H6" s="20" t="n"/>
       <c r="I6" s="20" t="n"/>
       <c r="J6" s="20" t="n"/>
@@ -1893,39 +1815,13 @@
       <c r="AY6" s="20" t="n"/>
     </row>
     <row r="7" ht="16.5" customHeight="1" s="37">
-      <c r="A7" s="20" t="inlineStr">
-        <is>
-          <t>25S02270004</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>PTseq</t>
-        </is>
-      </c>
-      <c r="C7" s="20" t="inlineStr">
-        <is>
-          <t>100K</t>
-        </is>
-      </c>
-      <c r="D7" s="27" t="inlineStr">
-        <is>
-          <t>鼻咽拭子</t>
-        </is>
-      </c>
-      <c r="E7" s="20" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F7" s="20" t="inlineStr">
-        <is>
-          <t>DNA+RNA</t>
-        </is>
-      </c>
-      <c r="G7" s="20" t="n">
-        <v>7</v>
-      </c>
+      <c r="A7" s="20" t="n"/>
+      <c r="B7" s="20" t="n"/>
+      <c r="C7" s="20" t="n"/>
+      <c r="D7" s="27" t="n"/>
+      <c r="E7" s="20" t="n"/>
+      <c r="F7" s="20" t="n"/>
+      <c r="G7" s="20" t="n"/>
       <c r="H7" s="20" t="n"/>
       <c r="I7" s="20" t="n"/>
       <c r="J7" s="20" t="n"/>
@@ -1958,39 +1854,13 @@
       <c r="AY7" s="20" t="n"/>
     </row>
     <row r="8" ht="16.5" customHeight="1" s="37">
-      <c r="A8" s="20" t="inlineStr">
-        <is>
-          <t>25S02270005</t>
-        </is>
-      </c>
-      <c r="B8" s="20" t="inlineStr">
-        <is>
-          <t>PTseq</t>
-        </is>
-      </c>
-      <c r="C8" s="20" t="inlineStr">
-        <is>
-          <t>100K</t>
-        </is>
-      </c>
-      <c r="D8" s="27" t="inlineStr">
-        <is>
-          <t>呼吸道其他</t>
-        </is>
-      </c>
-      <c r="E8" s="20" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F8" s="20" t="inlineStr">
-        <is>
-          <t>DNA+RNA</t>
-        </is>
-      </c>
-      <c r="G8" s="20" t="n">
-        <v>8</v>
-      </c>
+      <c r="A8" s="20" t="n"/>
+      <c r="B8" s="20" t="n"/>
+      <c r="C8" s="20" t="n"/>
+      <c r="D8" s="27" t="n"/>
+      <c r="E8" s="20" t="n"/>
+      <c r="F8" s="20" t="n"/>
+      <c r="G8" s="20" t="n"/>
       <c r="H8" s="20" t="n"/>
       <c r="I8" s="20" t="n"/>
       <c r="J8" s="20" t="n"/>
@@ -2023,39 +1893,13 @@
       <c r="AY8" s="20" t="n"/>
     </row>
     <row r="9" ht="16.5" customHeight="1" s="37">
-      <c r="A9" s="20" t="inlineStr">
-        <is>
-          <t>25S02270006</t>
-        </is>
-      </c>
-      <c r="B9" s="20" t="inlineStr">
-        <is>
-          <t>PTseq</t>
-        </is>
-      </c>
-      <c r="C9" s="20" t="inlineStr">
-        <is>
-          <t>100K</t>
-        </is>
-      </c>
-      <c r="D9" s="27" t="inlineStr">
-        <is>
-          <t>痰液</t>
-        </is>
-      </c>
-      <c r="E9" s="20" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F9" s="20" t="inlineStr">
-        <is>
-          <t>DNA+RNA</t>
-        </is>
-      </c>
-      <c r="G9" s="20" t="n">
-        <v>10</v>
-      </c>
+      <c r="A9" s="20" t="n"/>
+      <c r="B9" s="20" t="n"/>
+      <c r="C9" s="20" t="n"/>
+      <c r="D9" s="27" t="n"/>
+      <c r="E9" s="20" t="n"/>
+      <c r="F9" s="20" t="n"/>
+      <c r="G9" s="20" t="n"/>
       <c r="H9" s="20" t="n"/>
       <c r="I9" s="20" t="n"/>
       <c r="J9" s="20" t="n"/>
@@ -2105,7 +1949,7 @@
   </conditionalFormatting>
   <pageMargins left="0.31496062992126" right="0.31496062992126" top="0.748031496062992" bottom="0.748031496062992" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup orientation="landscape" paperSize="9" scale="29" fitToHeight="0"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <drawing ns1:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2404,7 +2248,7 @@
     <row r="4" ht="12.75" customHeight="1" s="37">
       <c r="A4" s="51" t="inlineStr">
         <is>
-          <t>25S02270001（示例）</t>
+          <t>26S08180001</t>
         </is>
       </c>
       <c r="B4" s="51" t="inlineStr">
@@ -2447,7 +2291,7 @@
       <c r="Q4" s="51" t="n"/>
       <c r="R4" s="51" t="inlineStr">
         <is>
-          <t>P20260123001</t>
+          <t>P20260818001</t>
         </is>
       </c>
       <c r="S4" s="53" t="inlineStr">
@@ -2457,8 +2301,16 @@
       </c>
       <c r="T4" s="51" t="n"/>
       <c r="U4" s="51" t="n"/>
-      <c r="V4" s="51" t="n"/>
-      <c r="W4" s="51" t="n"/>
+      <c r="V4" s="51" t="inlineStr">
+        <is>
+          <t>25B53569560</t>
+        </is>
+      </c>
+      <c r="W4" s="51" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
       <c r="X4" s="51" t="n"/>
       <c r="Y4" s="51" t="n"/>
       <c r="Z4" s="53" t="n"/>
@@ -2471,13 +2323,39 @@
       <c r="AG4" s="51" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1" s="37">
-      <c r="A5" s="54" t="n"/>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="54" t="n"/>
-      <c r="F5" s="54" t="n"/>
-      <c r="G5" s="54" t="n"/>
+      <c r="A5" s="54" t="inlineStr">
+        <is>
+          <t>26S08180002</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>PTseq</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>100K</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>痰液</t>
+        </is>
+      </c>
+      <c r="E5" s="54" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F5" s="54" t="inlineStr">
+        <is>
+          <t>DNA+RNA</t>
+        </is>
+      </c>
+      <c r="G5" s="54" t="n">
+        <v>2</v>
+      </c>
       <c r="H5" s="54" t="n"/>
       <c r="I5" s="54" t="n"/>
       <c r="J5" s="54" t="n"/>
@@ -2492,9 +2370,19 @@
       <c r="S5" s="3" t="n"/>
       <c r="T5" s="3" t="n"/>
       <c r="U5" s="54" t="n"/>
-      <c r="V5" s="3" t="n"/>
-      <c r="W5" s="3" t="n"/>
-      <c r="X5" s="3" t="n"/>
+      <c r="V5" s="3" t="inlineStr">
+        <is>
+          <t>25B53569561</t>
+        </is>
+      </c>
+      <c r="W5" s="3" t="inlineStr">
+        <is>
+          <t>B7</t>
+        </is>
+      </c>
+      <c r="X5" s="3" t="n">
+        <v>20</v>
+      </c>
       <c r="Y5" s="54" t="n"/>
       <c r="Z5" s="3" t="n"/>
       <c r="AA5" s="3" t="n"/>
@@ -2781,27 +2669,47 @@
       </c>
       <c r="R8" s="57" t="inlineStr">
         <is>
-          <t>全流程/前处理建库/仅提取/DNA流程必填,1-3块板</t>
+          <t>提取/全流程/前处理建库填写，单块板</t>
         </is>
       </c>
       <c r="S8" s="57" t="inlineStr">
         <is>
-          <t>全流程/前处理建库/仅提取/DNA流程必填，格式限A1</t>
+          <t>真实输入孔位A1-H6</t>
         </is>
       </c>
       <c r="V8" s="57" t="inlineStr">
         <is>
-          <t>上机前准备任务必填,1-4块板</t>
+          <t>填写计划或实际建库板号；单独上机前准备最多3块</t>
         </is>
       </c>
       <c r="W8" s="57" t="inlineStr">
         <is>
-          <t>上机前准备任务必填，格式限A1</t>
+          <t>真实文库产物孔位A7-H12</t>
         </is>
       </c>
       <c r="X8" s="59" t="inlineStr">
         <is>
-          <t>上机前准备任务必填，≥2ng/μL</t>
+          <t>全流程/前处理建库开始前不用填写，由定量结果回填；单独上机前准备必须填写实测浓度，≥1 ng/µL</t>
+        </is>
+      </c>
+      <c r="Z8" s="58" t="inlineStr">
+        <is>
+          <t>本产品没有杂交洗脱，不用填写</t>
+        </is>
+      </c>
+      <c r="AD8" s="58" t="inlineStr">
+        <is>
+          <t>由脚本运行后生成，任务导入时不用填写</t>
+        </is>
+      </c>
+      <c r="AE8" s="58" t="inlineStr">
+        <is>
+          <t>由脚本运行后生成，任务导入时不用填写</t>
+        </is>
+      </c>
+      <c r="AF8" s="58" t="inlineStr">
+        <is>
+          <t>由脚本运行后生成，任务导入时不用填写</t>
         </is>
       </c>
     </row>
@@ -2815,27 +2723,27 @@
       <c r="G9" s="58" t="n"/>
       <c r="R9" s="57" t="inlineStr">
         <is>
-          <t>全流程/前处理建库流程必填，1块板</t>
+          <t>提取/全流程/前处理建库必填</t>
         </is>
       </c>
       <c r="S9" s="57" t="inlineStr">
         <is>
-          <t>全流程/前处理建库流程必填，格式仅限A1</t>
+          <t>A1-H6</t>
         </is>
       </c>
       <c r="V9" s="57" t="inlineStr">
         <is>
-          <t>上机前准备任务必填,1-4块板</t>
+          <t>继续建库时填写</t>
         </is>
       </c>
       <c r="W9" s="57" t="inlineStr">
         <is>
-          <t>上机前准备任务必填，格式限A1</t>
+          <t>A7-H12</t>
         </is>
       </c>
       <c r="X9" s="57" t="inlineStr">
         <is>
-          <t>上机前准备任务必填，≥2ng/μL</t>
+          <t>建库运行前不填写</t>
         </is>
       </c>
     </row>
@@ -2853,47 +2761,31 @@
       <c r="O10" s="58" t="n"/>
       <c r="P10" s="58" t="n"/>
       <c r="Q10" s="58" t="n"/>
-      <c r="R10" s="57" t="inlineStr">
-        <is>
-          <t>全流程/前处理建库/前处理杂洗必填</t>
-        </is>
-      </c>
-      <c r="S10" s="57" t="inlineStr">
-        <is>
-          <t>全流程/前处理建库/前处理杂洗必填，格式仅限A1</t>
-        </is>
-      </c>
+      <c r="R10" s="57" t="n"/>
+      <c r="S10" s="57" t="n"/>
       <c r="V10" s="57" t="inlineStr">
         <is>
-          <t>杂交洗脱必填</t>
+          <t>单独上机前准备输入：实际建库板号</t>
         </is>
       </c>
       <c r="W10" s="57" t="inlineStr">
         <is>
-          <t>杂交洗脱必填，格式仅限A1</t>
+          <t>实际文库孔位A7-H12</t>
         </is>
       </c>
       <c r="X10" s="57" t="inlineStr">
         <is>
-          <t>杂交洗脱必填</t>
+          <t>实测浓度，≥1 ng/µL</t>
         </is>
       </c>
       <c r="Y10" s="58" t="n"/>
       <c r="Z10" s="58" t="inlineStr">
         <is>
-          <t>上机前准备必填</t>
-        </is>
-      </c>
-      <c r="AA10" s="58" t="inlineStr">
-        <is>
-          <t>上机前准备必填，格式仅限A1。同一杂交组内的样本孔位号均填写同一个</t>
-        </is>
-      </c>
-      <c r="AB10" s="58" t="inlineStr">
-        <is>
-          <t>上机前准备必填，≥10ng/μL。同一杂交组内的样本浓度填写同一个</t>
-        </is>
-      </c>
+          <t>本产品没有杂交洗脱，不用填写</t>
+        </is>
+      </c>
+      <c r="AA10" s="58" t="n"/>
+      <c r="AB10" s="58" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="37">
       <c r="A11" s="54" t="n"/>
@@ -2932,16 +2824,7 @@
     <row r="12" ht="39" customHeight="1" s="37">
       <c r="A12" s="60" t="inlineStr">
         <is>
-          <t>注释（PTseq 病原靶向高通量测序）：
-1、枚举值填写均区分大小写。
-2、产品名称：PTseq；检测项目：PTseq病原靶向高通量测序；分析参数：100K。
-3、PTseq 样本类型仅限呼吸道：痰液、肺泡灌洗液、口咽拭子、鼻咽拭子、呼吸道其他；对照样本：阴性对照、阳性对照、空白对照。
-4、质控类型 S、P、N、B 分别代表 样本、阳性、阴性、空白；空白/阴阳性对照均进入 pooling 并上机测序（污染监控）。
-5、核酸类型：DNA+RNA。
-6、BARCODE 按实际使用的编号填写（可不连续，例：1、2、5、7、8、10）。
-7、全流程 / 前处理建库：前处理孔位格式限 A1，单块前处理板。
-8、单独上机前准备：建库板号 1–3 块（对应 POS6/7/11）；建库孔位为真实产物孔，格式限 A7–H12；建库产物浓度必填，≥1 ng/µL（低于阈值将被剔除，不进 pooling）。
-9、PTseq 无杂交/杂洗步骤，杂交文库编号、杂洗相关列留空。</t>
+          <t>填写要求：提取/全流程/前处理建库填写前处理板号和前处理孔位；继续建库时填写计划建库板号和孔位。单独上机前准备填写实际建库板号、实际文库孔位和实测浓度。本产品没有杂交洗脱，相关内容不用填写。上机前准备板号、上机前准备孔位号和DNB浓度由脚本运行后生成，导入时不填写。</t>
         </is>
       </c>
       <c r="B12" s="61" t="n"/>

</xml_diff>

<commit_message>
fix(middleware): make PTseq route IDs unique
</commit_message>
<xml_diff>
--- a/中台配置/GenSIRO48-PTseq/Resources/SIRO48_template.xlsx
+++ b/中台配置/GenSIRO48-PTseq/Resources/SIRO48_template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="样本信息列表" sheetId="1" r:id="R3110a20a8ef74006"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="示例说明及编写要求" sheetId="2" r:id="Rebea0f9f4e8d4b17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="样本信息列表" sheetId="1" r:id="R222654f0aa9a416a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="示例说明及编写要求" sheetId="2" r:id="R453969153bb64f7d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1058,13 +1058,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="/xl/media/image1.jpeg"/>
+        <xdr:cNvPr id="1" name="/xl/media/image.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R78d6a456b27942a1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0368e86f8fcb40a7"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1871,7 +1871,7 @@
     <x:cfRule type="duplicateValues" dxfId="0" priority="4"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reead16d9c0b346cd"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra12e316bcf8f4fbd"/>
 </x:worksheet>
 </file>
 
@@ -2558,7 +2558,7 @@
         <x:v>仅上机前准备任务填写；最多 3 块文库板</x:v>
       </x:c>
       <x:c r="W9" s="57" t="str">
-        <x:v>多板按板号首次出现顺序对应 POS6、POS7、POS11</x:v>
+        <x:v>多板按板号首次出现顺序对应 POS6、POS11、POS7</x:v>
       </x:c>
       <x:c r="X9" s="57" t="str">
         <x:v>仅上机前准备任务填写</x:v>
@@ -2629,7 +2629,7 @@
         <x:v>PTseq 填写要求：
 1、所有任务填写样本编号、产品名称、分析参数、样本类型、质控类型、核酸类型和 BARCODE。产品名称为 PTseq，分析参数为 100K，核酸类型为 DNA+RNA。
 2、全流程和前处理建库任务同时填写前处理板号与前处理孔位。孔位按样本在样本架中的实际摆放填写；连续摆放时顺序为 A1、B1…H1、A2…，最多 48 个样本。
-3、上机前准备任务同时填写建库板号、建库孔位与实测建库产物浓度。最多 3 块文库板；板号按首次出现顺序对应 POS6、POS7、POS11。PTseq 建库产物默认位于 A7-H12，填写时以实际孔位为准。
+3、上机前准备任务同时填写建库板号、建库孔位与实测建库产物浓度。最多 3 块文库板；板号按首次出现顺序对应 POS6、POS11、POS7。PTseq 建库产物默认位于 A7-H12，填写时以实际孔位为准。
 4、质控类型 S、P、N、B 分别表示样本、阳性对照、阴性对照、空白对照。空白对照的孔位必须与实际摆放一致。
 5、PTseq 没有杂交/杂洗步骤。任务导入不使用的其余列留空。</x:v>
       </x:c>

</xml_diff>

<commit_message>
docs(middleware): document PTseq barcode order
</commit_message>
<xml_diff>
--- a/中台配置/GenSIRO48-PTseq/Resources/SIRO48_template.xlsx
+++ b/中台配置/GenSIRO48-PTseq/Resources/SIRO48_template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="样本信息列表" sheetId="1" r:id="R222654f0aa9a416a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="示例说明及编写要求" sheetId="2" r:id="R453969153bb64f7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="样本信息列表" sheetId="1" r:id="R7d539cf1a40143cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="示例说明及编写要求" sheetId="2" r:id="R5cd4a536d53e4f50"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1064,7 +1064,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0368e86f8fcb40a7"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rcddc3cd3fe4e4b47"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1871,7 +1871,7 @@
     <x:cfRule type="duplicateValues" dxfId="0" priority="4"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra12e316bcf8f4fbd"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ea69a4791c44067"/>
 </x:worksheet>
 </file>
 
@@ -2518,7 +2518,7 @@
         <x:v>DNA+RNA</x:v>
       </x:c>
       <x:c r="G8" s="59" t="str">
-        <x:v>按实际使用的 T6 Barcode 编号填写</x:v>
+        <x:v>不得按 1-48 连续填写；按本产品 T6 Barcode 固定顺序填写，完整顺序见下方说明</x:v>
       </x:c>
       <x:c r="H8" s="58"/>
       <x:c r="L8" s="23" t="str">
@@ -2631,7 +2631,8 @@
 2、全流程和前处理建库任务同时填写前处理板号与前处理孔位。孔位按样本在样本架中的实际摆放填写；连续摆放时顺序为 A1、B1…H1、A2…，最多 48 个样本。
 3、上机前准备任务同时填写建库板号、建库孔位与实测建库产物浓度。最多 3 块文库板；板号按首次出现顺序对应 POS6、POS11、POS7。PTseq 建库产物默认位于 A7-H12，填写时以实际孔位为准。
 4、质控类型 S、P、N、B 分别表示样本、阳性对照、阴性对照、空白对照。空白对照的孔位必须与实际摆放一致。
-5、PTseq 没有杂交/杂洗步骤。任务导入不使用的其余列留空。</x:v>
+5、PTseq 没有杂交/杂洗步骤。任务导入不使用的其余列留空。
+6、BARCODE 不得按 1-48 连续填写。48 个样本依次为：1、2、5、7、8、10、11、12、14、15、17、18、19、20、22、24、25、26、27、28、30、31、32、34、36、38、39、40、41、42、43、44、45、46、47、49、50、52、53、54、55、57、58、59、60、61、62、65。必须与实际使用的 T6 Barcode 一一对应，同一个 DNB 内不得出现重复 BARCODE。</x:v>
       </x:c>
       <x:c r="B12" s="61" t="n"/>
       <x:c r="C12" s="61" t="n"/>

</xml_diff>

<commit_message>
docs(middleware): align sequencing prep wells to A7-H12
</commit_message>
<xml_diff>
--- a/中台配置/GenSIRO48-PTseq/Resources/SIRO48_template.xlsx
+++ b/中台配置/GenSIRO48-PTseq/Resources/SIRO48_template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="样本信息列表" sheetId="1" r:id="R7d539cf1a40143cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="示例说明及编写要求" sheetId="2" r:id="R5cd4a536d53e4f50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="样本信息列表" sheetId="1" r:id="R72688f38ff18441b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="示例说明及编写要求" sheetId="2" r:id="R14628840b6944554"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1064,7 +1064,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rcddc3cd3fe4e4b47"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4fe73c1a6f8e4b81"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1871,7 +1871,7 @@
     <x:cfRule type="duplicateValues" dxfId="0" priority="4"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ea69a4791c44067"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6090e7c4ceea4cf0"/>
 </x:worksheet>
 </file>
 
@@ -2251,7 +2251,7 @@
         <x:v>L20260123001</x:v>
       </x:c>
       <x:c r="W5" s="3" t="str">
-        <x:v>B7</x:v>
+        <x:v>A7</x:v>
       </x:c>
       <x:c r="X5" s="3" t="n">
         <x:v>30</x:v>
@@ -2534,7 +2534,7 @@
         <x:v>填写实际建库产物板条码；同一块板使用同一板号</x:v>
       </x:c>
       <x:c r="W8" s="57" t="str">
-        <x:v>填写实际文库孔位；PTseq 建库产物默认位于 A7-H12</x:v>
+        <x:v>填写实际建库产物物理孔位；范围仅限 A7-H12</x:v>
       </x:c>
       <x:c r="X8" s="59" t="str">
         <x:v>填写实测建库产物浓度（ng/µL）；脚本筛选阈值为 1 ng/µL</x:v>
@@ -2558,7 +2558,7 @@
         <x:v>仅上机前准备任务填写；最多 3 块文库板</x:v>
       </x:c>
       <x:c r="W9" s="57" t="str">
-        <x:v>多板按板号首次出现顺序对应 POS6、POS11、POS7</x:v>
+        <x:v>连续摆放时依次 A7、B7…H7、A8…H12；多板按板号首次出现顺序对应 POS6、POS11、POS7</x:v>
       </x:c>
       <x:c r="X9" s="57" t="str">
         <x:v>仅上机前准备任务填写</x:v>
@@ -2629,7 +2629,7 @@
         <x:v>PTseq 填写要求：
 1、所有任务填写样本编号、产品名称、分析参数、样本类型、质控类型、核酸类型和 BARCODE。产品名称为 PTseq，分析参数为 100K，核酸类型为 DNA+RNA。
 2、全流程和前处理建库任务同时填写前处理板号与前处理孔位。孔位按样本在样本架中的实际摆放填写；连续摆放时顺序为 A1、B1…H1、A2…，最多 48 个样本。
-3、上机前准备任务同时填写建库板号、建库孔位与实测建库产物浓度。最多 3 块文库板；板号按首次出现顺序对应 POS6、POS11、POS7。PTseq 建库产物默认位于 A7-H12，填写时以实际孔位为准。
+3、上机前准备任务同时填写建库板号、建库孔位与实测建库产物浓度。最多 3 块文库板；板号按首次出现顺序对应 POS6、POS11、POS7。建库孔位必须填写实际物理孔位，范围仅限 A7-H12；连续摆放时顺序为 A7、B7…H7、A8…H12。
 4、质控类型 S、P、N、B 分别表示样本、阳性对照、阴性对照、空白对照。空白对照的孔位必须与实际摆放一致。
 5、PTseq 没有杂交/杂洗步骤。任务导入不使用的其余列留空。
 6、BARCODE 不得按 1-48 连续填写。48 个样本依次为：1、2、5、7、8、10、11、12、14、15、17、18、19、20、22、24、25、26、27、28、30、31、32、34、36、38、39、40、41、42、43、44、45、46、47、49、50、52、53、54、55、57、58、59、60、61、62、65。必须与实际使用的 T6 Barcode 一一对应，同一个 DNB 内不得出现重复 BARCODE。</x:v>

</xml_diff>

<commit_message>
docs(E25): align SOP and solution package records
</commit_message>
<xml_diff>
--- a/中台配置/GenSIRO48-PTseq/Resources/SIRO48_template.xlsx
+++ b/中台配置/GenSIRO48-PTseq/Resources/SIRO48_template.xlsx
@@ -2603,6 +2603,11 @@
           <t>全流程/前处理建库流程必填，格式仅限A1；按样本在样本架中的实际孔位填写，连续摆放时依次A1、B1…H1、A2…</t>
         </is>
       </c>
+      <c r="T8" s="68" t="inlineStr">
+        <is>
+          <t>适用于E25全流程；运行结束后由中台回填，导入任务时留空</t>
+        </is>
+      </c>
       <c r="V8" s="68" t="inlineStr">
         <is>
           <t>上机前准备任务必填，1-3块板；板号按首次出现顺序对应POS6、POS7、POS11</t>

</xml_diff>